<commit_message>
Files Updated for Imitator Backend
Signed-off-by: Alexandre Silva <alexandre.silva.0004@gmail.com>
</commit_message>
<xml_diff>
--- a/examples/hammer/hammer.xlsx
+++ b/examples/hammer/hammer.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10611"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jose/Documents/Research/projects/valu3s/wip/uppx/examples/hammer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F67C3CD7-FE4C-C64F-90F9-724FFE210B06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B81FB6E-8DFD-D644-925D-99A86BEB8086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="21200" windowHeight="12980" xr2:uid="{F23A7857-2A5B-744A-861E-37E01B360061}"/>
+    <workbookView xWindow="7600" yWindow="1800" windowWidth="21200" windowHeight="12980" xr2:uid="{F23A7857-2A5B-744A-861E-37E01B360061}"/>
   </bookViews>
   <sheets>
     <sheet name="@Configurations" sheetId="15" r:id="rId1"/>
-    <sheet name="@FeatureModel" sheetId="16" r:id="rId2"/>
-    <sheet name="@Channels" sheetId="12" r:id="rId3"/>
-    <sheet name="@Limits" sheetId="6" r:id="rId4"/>
-    <sheet name="&lt;queries&gt;" sheetId="14" r:id="rId5"/>
+    <sheet name="@Limits" sheetId="6" r:id="rId2"/>
+    <sheet name="&lt;queries&gt;" sheetId="14" r:id="rId3"/>
+    <sheet name="@FeatureModel" sheetId="16" r:id="rId4"/>
+    <sheet name="@Channels" sheetId="12" r:id="rId5"/>
     <sheet name="AvailableFunctions" sheetId="13" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -677,9 +677,6 @@
     <t>Count</t>
   </si>
   <si>
-    <t>CountNails</t>
-  </si>
-  <si>
     <t>would overflow "nails" when checking</t>
   </si>
   <si>
@@ -765,6 +762,9 @@
   </si>
   <si>
     <t>not needed</t>
+  </si>
+  <si>
+    <t>NormalCount</t>
   </si>
 </sst>
 </file>
@@ -1305,7 +1305,7 @@
         <v>210</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G1" s="9"/>
     </row>
@@ -1409,7 +1409,7 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>211</v>
+        <v>240</v>
       </c>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -1431,7 +1431,7 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>177</v>
@@ -1457,7 +1457,7 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -1626,175 +1626,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B5B459A-3BB1-EB4C-924B-0D3FED2B4C76}">
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="8.6640625" customWidth="1"/>
-    <col min="2" max="2" width="13.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
-        <v>221</v>
-      </c>
-      <c r="B1" s="15" t="s">
-        <v>236</v>
-      </c>
-      <c r="C1" s="15" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="14"/>
-      <c r="B2" s="15"/>
-      <c r="C2" s="16" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="13"/>
-      <c r="B3" s="15"/>
-      <c r="C3" s="17" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="13"/>
-      <c r="B4" s="18" t="s">
-        <v>237</v>
-      </c>
-      <c r="C4" s="18" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="13"/>
-      <c r="B5" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>210</v>
-      </c>
-      <c r="D5" s="20" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="12"/>
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="12" t="s">
-        <v>239</v>
-      </c>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="12" t="s">
-        <v>223</v>
-      </c>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="12" t="s">
-        <v>224</v>
-      </c>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B10" s="12"/>
-      <c r="C10" s="12"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="12"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="12" t="s">
-        <v>226</v>
-      </c>
-      <c r="D12" t="s">
-        <v>240</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B44A7D45-3D37-034F-A1FB-B28B84ABA07F}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="37.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="19" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>182</v>
-      </c>
-      <c r="C3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B4" t="s">
-        <v>182</v>
-      </c>
-      <c r="C4" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>183</v>
-      </c>
-      <c r="C6" t="s">
-        <v>185</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16772568-7503-3B4E-B82C-A26E56E7827F}">
   <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1830,7 +1661,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B3" s="5">
         <v>100</v>
@@ -1844,7 +1675,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B4" s="5">
         <v>50</v>
@@ -1861,7 +1692,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B5" s="2">
         <v>200</v>
@@ -1909,7 +1740,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B8" s="2">
         <v>0</v>
@@ -1918,29 +1749,29 @@
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E9" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B10" s="2" t="b">
         <v>0</v>
@@ -1949,12 +1780,12 @@
         <v>208</v>
       </c>
       <c r="E10" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B11" s="2" t="b">
         <v>1</v>
@@ -1963,10 +1794,10 @@
         <v>208</v>
       </c>
       <c r="D11" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E11" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -2026,7 +1857,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E766410-42AB-D842-913C-A2316B1EA100}">
   <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2054,10 +1885,10 @@
         <v>0</v>
       </c>
       <c r="D2" s="25" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E2" s="25" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -2071,7 +1902,7 @@
         <v>171</v>
       </c>
       <c r="E3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -2132,35 +1963,204 @@
         <v>200</v>
       </c>
       <c r="E8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="21" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B9" t="s">
         <v>210</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D9" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="21" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B10" t="s">
         <v>210</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D10" t="s">
-        <v>232</v>
+        <v>231</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B5B459A-3BB1-EB4C-924B-0D3FED2B4C76}">
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="8.6640625" customWidth="1"/>
+    <col min="2" max="2" width="13.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>235</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="14"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="16" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="13"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="17" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="13"/>
+      <c r="B4" s="18" t="s">
+        <v>236</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="13"/>
+      <c r="B5" s="19" t="s">
+        <v>221</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>210</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="12"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="12"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="12" t="s">
+        <v>238</v>
+      </c>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="B9" s="12"/>
+      <c r="C9" s="12"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B10" s="12"/>
+      <c r="C10" s="12"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="12"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="12" t="s">
+        <v>225</v>
+      </c>
+      <c r="D12" t="s">
+        <v>239</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B44A7D45-3D37-034F-A1FB-B28B84ABA07F}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="37.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>182</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B4" t="s">
+        <v>182</v>
+      </c>
+      <c r="C4" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>183</v>
+      </c>
+      <c r="C6" t="s">
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -2979,6 +2979,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DA12DE6878FEE740AAE11B8EF5A3BEB8" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ccf3f071624932fa9b6b142dc8790e1c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bf33d030-a745-437b-8efe-493a0e84c7f1" xmlns:ns3="38766943-c6ee-43fb-a1f1-f050a673c741" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="46fa4806b78295368f283e4cef5efe23" ns2:_="" ns3:_="">
     <xsd:import namespace="bf33d030-a745-437b-8efe-493a0e84c7f1"/>
@@ -3189,36 +3204,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{030D8A7F-6A3B-4D41-86D3-C760184B49E7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A07F53CA-6B4E-4B2E-8600-AB0859BD2077}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="bf33d030-a745-437b-8efe-493a0e84c7f1"/>
-    <ds:schemaRef ds:uri="38766943-c6ee-43fb-a1f1-f050a673c741"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3241,9 +3230,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A07F53CA-6B4E-4B2E-8600-AB0859BD2077}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{030D8A7F-6A3B-4D41-86D3-C760184B49E7}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="bf33d030-a745-437b-8efe-493a0e84c7f1"/>
+    <ds:schemaRef ds:uri="38766943-c6ee-43fb-a1f1-f050a673c741"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>